<commit_message>
v1.1: agrega operación potencia (CR-001) con ciclo for, pruebas y gestión del cambio
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KBDxQmfUDg5aQRniKn28Ls
</commit_message>
<xml_diff>
--- a/docs/Pruebas_Calculadora.xlsx
+++ b/docs/Pruebas_Calculadora.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1529,39 +1529,509 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>TC-23</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>potencia</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Potencia positiva</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>PASA</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
     <row r="25">
-      <c r="A25" t="inlineStr"/>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>TC-24</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>potencia</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Exponente cero</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>PASA</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>TC-25</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>potencia</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Exponente uno</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>PASA</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>TC-26</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>potencia</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Base negativa, exponente impar</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>-8</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>-8</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>PASA</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>TC-27</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>potencia</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Base negativa, exponente par</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>PASA</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>TC-28</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>potencia</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Base cero</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>PASA</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>TC-29</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>potencia</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Cero elevado a cero</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>PASA</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>TC-30</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>potencia</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Exponente negativo</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>-1</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>a ^ b -&gt; Error: el exponente debe ser mayor o igual a cero.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>a ^ b -&gt; Error: el exponente debe ser mayor o igual a cero.</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>PASA</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>TC-31</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>potencia</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Resultado demasiado grande</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>a ^ b -&gt; Error: el resultado de la potencia es demasiado grande.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>a ^ b -&gt; Error: el resultado de la potencia es demasiado grande.</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>PASA</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>TC-32</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>potencia</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Mayor potencia de 2 en long</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>4611686018427387904</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>4611686018427387904</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>PASA</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
         <is>
           <t>Total casos</t>
         </is>
       </c>
-      <c r="D25" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr"/>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr">
+      <c r="D35" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr">
         <is>
           <t>Pasan</t>
         </is>
       </c>
-      <c r="D26" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr"/>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr">
+      <c r="D36" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr">
         <is>
           <t>Fallan</t>
         </is>
       </c>
-      <c r="D27" t="n">
+      <c r="D37" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>